<commit_message>
Full info 950 products collected by establishing collection pipeline
</commit_message>
<xml_diff>
--- a/data/input/test_keywords.xlsx
+++ b/data/input/test_keywords.xlsx
@@ -1,16 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="48" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4354A7F-F0EA-4334-BF3D-65629C0C04E4}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\BJIT\Practical\Projects\Amazon-Marketplace-Product-Intelligence-Platform\data\input\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57C41EF7-44FC-4CF3-A9E4-3F69FFE45257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4245" yWindow="4245" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191028"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -130,7 +136,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -521,13 +527,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B29"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="37.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -535,7 +541,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -543,7 +549,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -551,7 +557,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -559,7 +565,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -567,7 +573,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -575,7 +581,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -583,7 +589,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -591,7 +597,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -599,7 +605,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -607,7 +613,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>11</v>
       </c>
@@ -615,7 +621,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>13</v>
       </c>
@@ -623,7 +629,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>14</v>
       </c>
@@ -631,7 +637,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>15</v>
       </c>
@@ -639,7 +645,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>16</v>
       </c>
@@ -647,7 +653,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>17</v>
       </c>
@@ -655,7 +661,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>18</v>
       </c>
@@ -663,7 +669,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>19</v>
       </c>
@@ -671,7 +677,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>20</v>
       </c>
@@ -679,7 +685,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>21</v>
       </c>
@@ -687,7 +693,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>22</v>
       </c>
@@ -695,7 +701,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>23</v>
       </c>
@@ -703,7 +709,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>24</v>
       </c>
@@ -711,7 +717,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>25</v>
       </c>
@@ -719,7 +725,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>26</v>
       </c>
@@ -727,7 +733,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>27</v>
       </c>
@@ -735,7 +741,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>28</v>
       </c>
@@ -743,7 +749,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="28" spans="1:2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>29</v>
       </c>
@@ -751,7 +757,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="29" spans="1:2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>30</v>
       </c>

</xml_diff>